<commit_message>
corregidas unidades, se movio iWUE a cleaning asi como add info site
</commit_message>
<xml_diff>
--- a/Results_isofys/NUMEX_cellulose_C13-10042025_results.xlsx
+++ b/Results_isofys/NUMEX_cellulose_C13-10042025_results.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\selene.baez\Downloads\NUMEX preliminary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\selene.baez\Downloads\NUMEX_preliminar\Results_isofys\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="389">
   <si>
     <t>site</t>
   </si>
@@ -957,264 +957,129 @@
     <t>Erythrina edulis</t>
   </si>
   <si>
-    <t>41.50%</t>
-  </si>
-  <si>
-    <t>44.05%</t>
-  </si>
-  <si>
     <t>-30.69</t>
   </si>
   <si>
-    <t>43.49%</t>
-  </si>
-  <si>
     <t>-30.99</t>
   </si>
   <si>
-    <t>42.61%</t>
-  </si>
-  <si>
     <t>-32.02</t>
   </si>
   <si>
-    <t>42.84%</t>
-  </si>
-  <si>
     <t>-30.83</t>
   </si>
   <si>
-    <t>43.55%</t>
-  </si>
-  <si>
     <t>-32.15</t>
   </si>
   <si>
-    <t>44.19%</t>
-  </si>
-  <si>
     <t>-31.96</t>
   </si>
   <si>
-    <t>43.81%</t>
-  </si>
-  <si>
     <t>-29.72</t>
   </si>
   <si>
-    <t>44.90%</t>
-  </si>
-  <si>
     <t>-33.09</t>
   </si>
   <si>
-    <t>41.66%</t>
-  </si>
-  <si>
     <t>-29.29</t>
   </si>
   <si>
-    <t>43.20%</t>
-  </si>
-  <si>
     <t>-28.42</t>
   </si>
   <si>
-    <t>42.45%</t>
-  </si>
-  <si>
     <t>-30.43</t>
   </si>
   <si>
-    <t>42.05%</t>
-  </si>
-  <si>
     <t>-30.26</t>
   </si>
   <si>
-    <t>36.70%</t>
-  </si>
-  <si>
     <t>-30.98</t>
   </si>
   <si>
-    <t>38.95%</t>
-  </si>
-  <si>
     <t>-31.19</t>
   </si>
   <si>
-    <t>43.72%</t>
-  </si>
-  <si>
     <t>-29.28</t>
   </si>
   <si>
     <t>-31.98</t>
   </si>
   <si>
-    <t>42.33%</t>
-  </si>
-  <si>
     <t>-32.67</t>
   </si>
   <si>
-    <t>42.23%</t>
-  </si>
-  <si>
     <t>-32.01</t>
   </si>
   <si>
-    <t>42.00%</t>
-  </si>
-  <si>
-    <t>42.24%</t>
-  </si>
-  <si>
     <t>-30.01</t>
   </si>
   <si>
-    <t>42.21%</t>
-  </si>
-  <si>
     <t>-31.46</t>
   </si>
   <si>
     <t>-31.62</t>
   </si>
   <si>
-    <t>43.43%</t>
-  </si>
-  <si>
     <t>-30.74</t>
   </si>
   <si>
-    <t>41.42%</t>
-  </si>
-  <si>
-    <t>39.77%</t>
-  </si>
-  <si>
     <t>-28.20</t>
   </si>
   <si>
-    <t>42.28%</t>
-  </si>
-  <si>
     <t>-32.96</t>
   </si>
   <si>
-    <t>42.74%</t>
-  </si>
-  <si>
     <t>-32.93</t>
   </si>
   <si>
-    <t>42.37%</t>
-  </si>
-  <si>
     <t>-30.13</t>
   </si>
   <si>
-    <t>43.19%</t>
-  </si>
-  <si>
     <t>-30.91</t>
   </si>
   <si>
-    <t>42.17%</t>
-  </si>
-  <si>
     <t>-30.92</t>
   </si>
   <si>
-    <t>41.56%</t>
-  </si>
-  <si>
-    <t>43.27%</t>
-  </si>
-  <si>
     <t>-31.13</t>
   </si>
   <si>
-    <t>43.01%</t>
-  </si>
-  <si>
     <t>-31.33</t>
   </si>
   <si>
-    <t>41.89%</t>
-  </si>
-  <si>
     <t>-33.43</t>
   </si>
   <si>
-    <t>44.14%</t>
-  </si>
-  <si>
-    <t>42.27%</t>
-  </si>
-  <si>
     <t>-31.40</t>
   </si>
   <si>
-    <t>42.69%</t>
-  </si>
-  <si>
     <t>-30.05</t>
   </si>
   <si>
-    <t>43.36%</t>
-  </si>
-  <si>
     <t>-31.35</t>
   </si>
   <si>
-    <t>43.21%</t>
-  </si>
-  <si>
     <t>-31.76</t>
   </si>
   <si>
-    <t>42.87%</t>
-  </si>
-  <si>
     <t>-29.37</t>
   </si>
   <si>
-    <t>42.99%</t>
-  </si>
-  <si>
     <t>-30.34</t>
   </si>
   <si>
-    <t>42.50%</t>
-  </si>
-  <si>
     <t>-31.07</t>
   </si>
   <si>
-    <t>43.85%</t>
-  </si>
-  <si>
     <t>-30.54</t>
   </si>
   <si>
-    <t>38.08%</t>
-  </si>
-  <si>
     <t>-31.11</t>
   </si>
   <si>
-    <t>40.86%</t>
-  </si>
-  <si>
     <t>-29.19</t>
   </si>
   <si>
-    <t>35.73%</t>
-  </si>
-  <si>
     <t>-30.93</t>
   </si>
   <si>
@@ -1224,21 +1089,12 @@
     <t>-23.39</t>
   </si>
   <si>
-    <t>44.25%</t>
-  </si>
-  <si>
     <t>-31.09</t>
   </si>
   <si>
-    <t>39.84%</t>
-  </si>
-  <si>
     <t>-27.67</t>
   </si>
   <si>
-    <t>42.68%</t>
-  </si>
-  <si>
     <t>-25.47</t>
   </si>
   <si>
@@ -1248,126 +1104,69 @@
     <t>-26.58</t>
   </si>
   <si>
-    <t>43.63%</t>
-  </si>
-  <si>
     <t>-29.06</t>
   </si>
   <si>
-    <t>46.28%</t>
-  </si>
-  <si>
     <t>-27.23</t>
   </si>
   <si>
-    <t>45.46%</t>
-  </si>
-  <si>
     <t>-26.38</t>
   </si>
   <si>
-    <t>43.93%</t>
-  </si>
-  <si>
     <t>-25.70</t>
   </si>
   <si>
     <t>-25.65</t>
   </si>
   <si>
-    <t>45.73%</t>
-  </si>
-  <si>
     <t>-27.80</t>
   </si>
   <si>
-    <t>40.31%</t>
-  </si>
-  <si>
     <t>-25.51</t>
   </si>
   <si>
-    <t>43.60%</t>
-  </si>
-  <si>
     <t>-26.99</t>
   </si>
   <si>
     <t>-27.59</t>
   </si>
   <si>
-    <t>43.76%</t>
-  </si>
-  <si>
     <t>-24.53</t>
   </si>
   <si>
-    <t>44.46%</t>
-  </si>
-  <si>
     <t>-28.06</t>
   </si>
   <si>
-    <t>45.00%</t>
-  </si>
-  <si>
     <t>-23.86</t>
   </si>
   <si>
     <t>-29.10</t>
   </si>
   <si>
-    <t>44.59%</t>
-  </si>
-  <si>
     <t>-26.57</t>
   </si>
   <si>
-    <t>45.91%</t>
-  </si>
-  <si>
     <t>-29.76</t>
   </si>
   <si>
-    <t>40.08%</t>
-  </si>
-  <si>
     <t>-26.93</t>
   </si>
   <si>
-    <t>43.80%</t>
-  </si>
-  <si>
     <t>-28.09</t>
   </si>
   <si>
-    <t>43.50%</t>
-  </si>
-  <si>
     <t>-24.88</t>
   </si>
   <si>
-    <t>45.97%</t>
-  </si>
-  <si>
     <t>-26.80</t>
   </si>
   <si>
-    <t>43.66%</t>
-  </si>
-  <si>
     <t>-28.27</t>
   </si>
   <si>
-    <t>43.59%</t>
-  </si>
-  <si>
     <t>-28.85</t>
   </si>
   <si>
-    <t>43.71%</t>
-  </si>
-  <si>
     <t>-26.52</t>
   </si>
   <si>
@@ -1380,52 +1179,22 @@
     <t>-29.59</t>
   </si>
   <si>
-    <t>43.16%</t>
-  </si>
-  <si>
     <t>-26.37</t>
   </si>
   <si>
-    <t>47.75%</t>
-  </si>
-  <si>
     <t>-27.45</t>
   </si>
   <si>
-    <t>41.99%</t>
-  </si>
-  <si>
     <t>-28.47</t>
   </si>
   <si>
-    <t>42.98%</t>
-  </si>
-  <si>
     <t>-27.83</t>
   </si>
   <si>
-    <t>41.85%</t>
-  </si>
-  <si>
     <t>-28.73</t>
   </si>
   <si>
-    <t>42.73%</t>
-  </si>
-  <si>
-    <t>42.13%</t>
-  </si>
-  <si>
     <t>-27.57</t>
-  </si>
-  <si>
-    <t>42.81%</t>
-  </si>
-  <si>
-    <t>-28.13</t>
-  </si>
-  <si>
-    <t>43.91%</t>
   </si>
   <si>
     <t>[C]</t>
@@ -1649,7 +1418,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1694,17 +1463,20 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4327,19 +4099,19 @@
   <dimension ref="B1:E88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="8.7109375" style="20"/>
+    <col min="4" max="4" width="8.7109375" style="28"/>
     <col min="5" max="5" width="15.42578125" style="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="C1" t="s">
-        <v>465</v>
-      </c>
-      <c r="D1" s="20" t="s">
-        <v>462</v>
-      </c>
-      <c r="E1" s="24" t="s">
-        <v>463</v>
+        <v>388</v>
+      </c>
+      <c r="D1" s="28" t="s">
+        <v>385</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="2" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4349,11 +4121,11 @@
       <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="22" t="s">
-        <v>461</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>460</v>
+      <c r="D2" s="29">
+        <v>43.91</v>
+      </c>
+      <c r="E2" s="21">
+        <v>-28.13</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4363,11 +4135,11 @@
       <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="22" t="s">
-        <v>459</v>
+      <c r="D3" s="29">
+        <v>42.81</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>458</v>
+        <v>384</v>
       </c>
     </row>
     <row r="4" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4377,11 +4149,11 @@
       <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="22" t="s">
-        <v>457</v>
+      <c r="D4" s="29">
+        <v>42.13</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>445</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4391,11 +4163,11 @@
       <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="22" t="s">
-        <v>456</v>
+      <c r="D5" s="29">
+        <v>42.73</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>455</v>
+        <v>383</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4405,11 +4177,11 @@
       <c r="C6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="22" t="s">
-        <v>454</v>
+      <c r="D6" s="29">
+        <v>41.85</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>453</v>
+        <v>382</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4419,11 +4191,11 @@
       <c r="C7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="22" t="s">
-        <v>452</v>
+      <c r="D7" s="29">
+        <v>42.98</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>451</v>
+        <v>381</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4433,11 +4205,11 @@
       <c r="C8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="22" t="s">
-        <v>450</v>
+      <c r="D8" s="29">
+        <v>41.99</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>449</v>
+        <v>380</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4447,11 +4219,11 @@
       <c r="C9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="22" t="s">
-        <v>448</v>
+      <c r="D9" s="29">
+        <v>47.75</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>447</v>
+        <v>379</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4461,11 +4233,11 @@
       <c r="C10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="22" t="s">
-        <v>446</v>
+      <c r="D10" s="29">
+        <v>43.16</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>445</v>
+        <v>378</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4475,11 +4247,11 @@
       <c r="C11" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="22" t="s">
-        <v>415</v>
+      <c r="D11" s="29">
+        <v>43.6</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>444</v>
+        <v>377</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4489,11 +4261,11 @@
       <c r="C12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="22" t="s">
-        <v>341</v>
+      <c r="D12" s="29">
+        <v>42</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>443</v>
+        <v>376</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4503,11 +4275,11 @@
       <c r="C13" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="22" t="s">
-        <v>324</v>
+      <c r="D13" s="29">
+        <v>43.2</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>442</v>
+        <v>375</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4517,11 +4289,11 @@
       <c r="C14" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="22" t="s">
-        <v>441</v>
+      <c r="D14" s="29">
+        <v>43.71</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>440</v>
+        <v>374</v>
       </c>
     </row>
     <row r="15" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4531,11 +4303,11 @@
       <c r="C15" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="22" t="s">
-        <v>439</v>
+      <c r="D15" s="29">
+        <v>43.59</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>438</v>
+        <v>373</v>
       </c>
     </row>
     <row r="16" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4545,11 +4317,11 @@
       <c r="C16" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="22" t="s">
-        <v>437</v>
+      <c r="D16" s="29">
+        <v>43.66</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>436</v>
+        <v>372</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4559,11 +4331,11 @@
       <c r="C17" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D17" s="22" t="s">
-        <v>435</v>
+      <c r="D17" s="29">
+        <v>45.97</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>434</v>
+        <v>371</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4573,11 +4345,11 @@
       <c r="C18" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="22" t="s">
-        <v>433</v>
+      <c r="D18" s="29">
+        <v>43.5</v>
       </c>
       <c r="E18" s="21" t="s">
-        <v>432</v>
+        <v>370</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4587,11 +4359,11 @@
       <c r="C19" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D19" s="22" t="s">
-        <v>431</v>
+      <c r="D19" s="29">
+        <v>43.8</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>430</v>
+        <v>369</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4601,11 +4373,11 @@
       <c r="C20" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D20" s="22" t="s">
-        <v>429</v>
+      <c r="D20" s="29">
+        <v>40.08</v>
       </c>
       <c r="E20" s="21" t="s">
-        <v>428</v>
+        <v>368</v>
       </c>
     </row>
     <row r="21" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4615,11 +4387,11 @@
       <c r="C21" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D21" s="22" t="s">
-        <v>427</v>
+      <c r="D21" s="29">
+        <v>45.91</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>426</v>
+        <v>367</v>
       </c>
     </row>
     <row r="22" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4629,11 +4401,11 @@
       <c r="C22" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D22" s="22" t="s">
-        <v>425</v>
+      <c r="D22" s="29">
+        <v>44.59</v>
       </c>
       <c r="E22" s="21" t="s">
-        <v>424</v>
+        <v>366</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4643,11 +4415,11 @@
       <c r="C23" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D23" s="22" t="s">
-        <v>422</v>
+      <c r="D23" s="29">
+        <v>45</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>423</v>
+        <v>365</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4657,11 +4429,11 @@
       <c r="C24" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D24" s="22" t="s">
-        <v>422</v>
+      <c r="D24" s="29">
+        <v>45</v>
       </c>
       <c r="E24" s="21" t="s">
-        <v>421</v>
+        <v>364</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4671,11 +4443,11 @@
       <c r="C25" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D25" s="22" t="s">
-        <v>420</v>
+      <c r="D25" s="29">
+        <v>44.46</v>
       </c>
       <c r="E25" s="21" t="s">
-        <v>419</v>
+        <v>363</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4685,11 +4457,11 @@
       <c r="C26" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D26" s="22" t="s">
-        <v>418</v>
+      <c r="D26" s="29">
+        <v>43.76</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>417</v>
+        <v>362</v>
       </c>
     </row>
     <row r="27" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4699,11 +4471,11 @@
       <c r="C27" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D27" s="22" t="s">
-        <v>306</v>
+      <c r="D27" s="29">
+        <v>44.05</v>
       </c>
       <c r="E27" s="21" t="s">
-        <v>416</v>
+        <v>361</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4713,11 +4485,11 @@
       <c r="C28" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D28" s="22" t="s">
-        <v>415</v>
+      <c r="D28" s="29">
+        <v>43.6</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>414</v>
+        <v>360</v>
       </c>
     </row>
     <row r="29" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4727,11 +4499,11 @@
       <c r="C29" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D29" s="22" t="s">
-        <v>413</v>
+      <c r="D29" s="29">
+        <v>40.31</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>412</v>
+        <v>359</v>
       </c>
     </row>
     <row r="30" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4741,11 +4513,11 @@
       <c r="C30" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D30" s="22" t="s">
-        <v>306</v>
+      <c r="D30" s="29">
+        <v>44.05</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>409</v>
+        <v>357</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4755,11 +4527,11 @@
       <c r="C31" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D31" s="22" t="s">
-        <v>411</v>
+      <c r="D31" s="29">
+        <v>45.73</v>
       </c>
       <c r="E31" s="21" t="s">
-        <v>410</v>
+        <v>358</v>
       </c>
     </row>
     <row r="32" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4769,11 +4541,11 @@
       <c r="C32" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D32" s="22" t="s">
-        <v>334</v>
+      <c r="D32" s="29">
+        <v>43.72</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>409</v>
+        <v>357</v>
       </c>
     </row>
     <row r="33" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4783,11 +4555,11 @@
       <c r="C33" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D33" s="22" t="s">
-        <v>408</v>
+      <c r="D33" s="29">
+        <v>43.93</v>
       </c>
       <c r="E33" s="21" t="s">
-        <v>407</v>
+        <v>356</v>
       </c>
     </row>
     <row r="34" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4797,11 +4569,11 @@
       <c r="C34" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D34" s="22" t="s">
-        <v>406</v>
+      <c r="D34" s="29">
+        <v>45.46</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>405</v>
+        <v>355</v>
       </c>
     </row>
     <row r="35" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4811,11 +4583,11 @@
       <c r="C35" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D35" s="22" t="s">
-        <v>404</v>
+      <c r="D35" s="29">
+        <v>46.28</v>
       </c>
       <c r="E35" s="21" t="s">
-        <v>403</v>
+        <v>354</v>
       </c>
     </row>
     <row r="36" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4825,11 +4597,11 @@
       <c r="C36" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D36" s="22" t="s">
-        <v>402</v>
+      <c r="D36" s="29">
+        <v>43.63</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>401</v>
+        <v>353</v>
       </c>
     </row>
     <row r="37" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4839,11 +4611,11 @@
       <c r="C37" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="D37" s="22" t="s">
-        <v>374</v>
+      <c r="D37" s="29">
+        <v>43.36</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>400</v>
+        <v>352</v>
       </c>
     </row>
     <row r="38" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4853,11 +4625,11 @@
       <c r="C38" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D38" s="22" t="s">
-        <v>358</v>
+      <c r="D38" s="29">
+        <v>43.19</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>399</v>
+        <v>351</v>
       </c>
     </row>
     <row r="39" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4867,11 +4639,11 @@
       <c r="C39" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="D39" s="22" t="s">
-        <v>398</v>
+      <c r="D39" s="29">
+        <v>42.68</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>397</v>
+        <v>350</v>
       </c>
     </row>
     <row r="40" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4881,11 +4653,11 @@
       <c r="C40" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D40" s="22" t="s">
-        <v>396</v>
+      <c r="D40" s="29">
+        <v>39.840000000000003</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>395</v>
+        <v>349</v>
       </c>
     </row>
     <row r="41" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4895,11 +4667,11 @@
       <c r="C41" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D41" s="22" t="s">
-        <v>394</v>
+      <c r="D41" s="29">
+        <v>44.25</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>393</v>
+        <v>348</v>
       </c>
     </row>
     <row r="42" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4909,11 +4681,11 @@
       <c r="C42" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D42" s="22" t="s">
-        <v>328</v>
+      <c r="D42" s="29">
+        <v>42.05</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>392</v>
+        <v>347</v>
       </c>
     </row>
     <row r="43" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4923,11 +4695,11 @@
       <c r="C43" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D43" s="22" t="s">
-        <v>354</v>
+      <c r="D43" s="29">
+        <v>42.74</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>391</v>
+        <v>346</v>
       </c>
     </row>
     <row r="44" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4937,11 +4709,11 @@
       <c r="C44" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="D44" s="22" t="s">
-        <v>390</v>
+      <c r="D44" s="29">
+        <v>35.729999999999997</v>
       </c>
       <c r="E44" s="21" t="s">
-        <v>389</v>
+        <v>345</v>
       </c>
     </row>
     <row r="45" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4951,11 +4723,11 @@
       <c r="C45" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D45" s="22" t="s">
-        <v>388</v>
+      <c r="D45" s="29">
+        <v>40.86</v>
       </c>
       <c r="E45" s="21" t="s">
-        <v>387</v>
+        <v>344</v>
       </c>
     </row>
     <row r="46" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4965,11 +4737,11 @@
       <c r="C46" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="D46" s="22" t="s">
-        <v>386</v>
+      <c r="D46" s="29">
+        <v>38.08</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>385</v>
+        <v>343</v>
       </c>
     </row>
     <row r="47" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4979,11 +4751,11 @@
       <c r="C47" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="D47" s="22" t="s">
-        <v>384</v>
+      <c r="D47" s="29">
+        <v>43.85</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>383</v>
+        <v>342</v>
       </c>
     </row>
     <row r="48" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -4993,11 +4765,11 @@
       <c r="C48" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="D48" s="22" t="s">
-        <v>382</v>
+      <c r="D48" s="29">
+        <v>42.5</v>
       </c>
       <c r="E48" s="21" t="s">
-        <v>381</v>
+        <v>341</v>
       </c>
     </row>
     <row r="49" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5007,11 +4779,11 @@
       <c r="C49" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="D49" s="22" t="s">
-        <v>380</v>
+      <c r="D49" s="29">
+        <v>42.99</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>379</v>
+        <v>340</v>
       </c>
     </row>
     <row r="50" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5021,11 +4793,11 @@
       <c r="C50" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D50" s="22" t="s">
-        <v>378</v>
+      <c r="D50" s="29">
+        <v>42.87</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>377</v>
+        <v>339</v>
       </c>
     </row>
     <row r="51" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5035,11 +4807,11 @@
       <c r="C51" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D51" s="22" t="s">
-        <v>376</v>
+      <c r="D51" s="29">
+        <v>43.21</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>375</v>
+        <v>338</v>
       </c>
     </row>
     <row r="52" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5049,11 +4821,11 @@
       <c r="C52" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D52" s="22" t="s">
-        <v>374</v>
+      <c r="D52" s="29">
+        <v>43.36</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>373</v>
+        <v>337</v>
       </c>
     </row>
     <row r="53" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5063,11 +4835,11 @@
       <c r="C53" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D53" s="22" t="s">
-        <v>372</v>
+      <c r="D53" s="29">
+        <v>42.69</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>371</v>
+        <v>336</v>
       </c>
     </row>
     <row r="54" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5077,11 +4849,11 @@
       <c r="C54" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D54" s="22" t="s">
-        <v>370</v>
+      <c r="D54" s="29">
+        <v>42.27</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5091,11 +4863,11 @@
       <c r="C55" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D55" s="22" t="s">
-        <v>369</v>
+      <c r="D55" s="29">
+        <v>44.14</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>368</v>
+        <v>335</v>
       </c>
     </row>
     <row r="56" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5105,11 +4877,11 @@
       <c r="C56" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D56" s="22" t="s">
-        <v>367</v>
+      <c r="D56" s="29">
+        <v>41.89</v>
       </c>
       <c r="E56" s="21" t="s">
-        <v>366</v>
+        <v>334</v>
       </c>
     </row>
     <row r="57" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5119,11 +4891,11 @@
       <c r="C57" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D57" s="22" t="s">
-        <v>365</v>
+      <c r="D57" s="29">
+        <v>43.01</v>
       </c>
       <c r="E57" s="21" t="s">
-        <v>364</v>
+        <v>333</v>
       </c>
     </row>
     <row r="58" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5133,11 +4905,11 @@
       <c r="C58" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D58" s="22" t="s">
-        <v>363</v>
+      <c r="D58" s="29">
+        <v>43.27</v>
       </c>
       <c r="E58" s="21" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="59" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5147,11 +4919,11 @@
       <c r="C59" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D59" s="22" t="s">
-        <v>362</v>
+      <c r="D59" s="29">
+        <v>41.56</v>
       </c>
       <c r="E59" s="21" t="s">
-        <v>361</v>
+        <v>332</v>
       </c>
     </row>
     <row r="60" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5161,11 +4933,11 @@
       <c r="C60" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D60" s="22" t="s">
-        <v>360</v>
+      <c r="D60" s="29">
+        <v>42.17</v>
       </c>
       <c r="E60" s="21" t="s">
-        <v>359</v>
+        <v>331</v>
       </c>
     </row>
     <row r="61" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5175,11 +4947,11 @@
       <c r="C61" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D61" s="22" t="s">
-        <v>358</v>
+      <c r="D61" s="29">
+        <v>43.19</v>
       </c>
       <c r="E61" s="21" t="s">
-        <v>357</v>
+        <v>330</v>
       </c>
     </row>
     <row r="62" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5189,11 +4961,11 @@
       <c r="C62" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D62" s="22" t="s">
-        <v>356</v>
+      <c r="D62" s="29">
+        <v>42.37</v>
       </c>
       <c r="E62" s="21" t="s">
-        <v>355</v>
+        <v>329</v>
       </c>
     </row>
     <row r="63" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5203,11 +4975,11 @@
       <c r="C63" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D63" s="22" t="s">
-        <v>354</v>
+      <c r="D63" s="29">
+        <v>42.74</v>
       </c>
       <c r="E63" s="21" t="s">
-        <v>353</v>
+        <v>328</v>
       </c>
     </row>
     <row r="64" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5217,11 +4989,11 @@
       <c r="C64" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D64" s="22" t="s">
-        <v>352</v>
+      <c r="D64" s="29">
+        <v>42.28</v>
       </c>
       <c r="E64" s="21" t="s">
-        <v>351</v>
+        <v>327</v>
       </c>
     </row>
     <row r="65" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5231,11 +5003,11 @@
       <c r="C65" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D65" s="22" t="s">
-        <v>350</v>
+      <c r="D65" s="29">
+        <v>39.770000000000003</v>
       </c>
       <c r="E65" s="21" t="s">
-        <v>331</v>
+        <v>317</v>
       </c>
     </row>
     <row r="66" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5245,11 +5017,11 @@
       <c r="C66" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D66" s="22" t="s">
-        <v>349</v>
+      <c r="D66" s="29">
+        <v>41.42</v>
       </c>
       <c r="E66" s="21" t="s">
-        <v>348</v>
+        <v>326</v>
       </c>
     </row>
     <row r="67" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5259,11 +5031,11 @@
       <c r="C67" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D67" s="22" t="s">
-        <v>347</v>
+      <c r="D67" s="29">
+        <v>43.43</v>
       </c>
       <c r="E67" s="21" t="s">
-        <v>346</v>
+        <v>325</v>
       </c>
     </row>
     <row r="68" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5273,11 +5045,11 @@
       <c r="C68" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D68" s="22" t="s">
-        <v>305</v>
+      <c r="D68" s="29">
+        <v>41.5</v>
       </c>
       <c r="E68" s="21" t="s">
-        <v>345</v>
+        <v>324</v>
       </c>
     </row>
     <row r="69" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5287,11 +5059,11 @@
       <c r="C69" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D69" s="22" t="s">
-        <v>344</v>
+      <c r="D69" s="29">
+        <v>42.21</v>
       </c>
       <c r="E69" s="21" t="s">
-        <v>343</v>
+        <v>323</v>
       </c>
     </row>
     <row r="70" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5301,11 +5073,11 @@
       <c r="C70" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D70" s="22" t="s">
-        <v>342</v>
+      <c r="D70" s="29">
+        <v>42.24</v>
       </c>
       <c r="E70" s="21" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
     </row>
     <row r="71" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5315,11 +5087,11 @@
       <c r="C71" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D71" s="22" t="s">
-        <v>341</v>
+      <c r="D71" s="29">
+        <v>42</v>
       </c>
       <c r="E71" s="21" t="s">
-        <v>340</v>
+        <v>322</v>
       </c>
     </row>
     <row r="72" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5329,11 +5101,11 @@
       <c r="C72" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D72" s="22" t="s">
-        <v>339</v>
+      <c r="D72" s="29">
+        <v>42.23</v>
       </c>
       <c r="E72" s="21" t="s">
-        <v>338</v>
+        <v>321</v>
       </c>
     </row>
     <row r="73" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5343,11 +5115,11 @@
       <c r="C73" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D73" s="22" t="s">
-        <v>337</v>
+      <c r="D73" s="29">
+        <v>42.33</v>
       </c>
       <c r="E73" s="21" t="s">
-        <v>336</v>
+        <v>320</v>
       </c>
     </row>
     <row r="74" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5357,11 +5129,11 @@
       <c r="C74" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D74" s="22" t="s">
-        <v>314</v>
+      <c r="D74" s="29">
+        <v>43.55</v>
       </c>
       <c r="E74" s="21" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
     </row>
     <row r="75" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5371,11 +5143,11 @@
       <c r="C75" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D75" s="22" t="s">
-        <v>334</v>
+      <c r="D75" s="29">
+        <v>43.72</v>
       </c>
       <c r="E75" s="21" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="76" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5385,11 +5157,11 @@
       <c r="C76" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D76" s="22" t="s">
-        <v>332</v>
+      <c r="D76" s="29">
+        <v>38.950000000000003</v>
       </c>
       <c r="E76" s="21" t="s">
-        <v>331</v>
+        <v>317</v>
       </c>
     </row>
     <row r="77" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5399,25 +5171,25 @@
       <c r="C77" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D77" s="22" t="s">
-        <v>330</v>
+      <c r="D77" s="29">
+        <v>36.700000000000003</v>
       </c>
       <c r="E77" s="21" t="s">
-        <v>329</v>
+        <v>316</v>
       </c>
     </row>
     <row r="78" spans="2:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B78" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C78" s="23" t="s">
+      <c r="C78" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="D78" s="22" t="s">
-        <v>328</v>
+      <c r="D78" s="29">
+        <v>42.05</v>
       </c>
       <c r="E78" s="21" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
     </row>
     <row r="79" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5427,11 +5199,11 @@
       <c r="C79" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D79" s="22" t="s">
-        <v>326</v>
+      <c r="D79" s="29">
+        <v>42.45</v>
       </c>
       <c r="E79" s="21" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
     </row>
     <row r="80" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5441,11 +5213,11 @@
       <c r="C80" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D80" s="22" t="s">
-        <v>324</v>
+      <c r="D80" s="29">
+        <v>43.2</v>
       </c>
       <c r="E80" s="21" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
     </row>
     <row r="81" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5455,11 +5227,11 @@
       <c r="C81" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D81" s="22" t="s">
-        <v>322</v>
+      <c r="D81" s="29">
+        <v>41.66</v>
       </c>
       <c r="E81" s="21" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
     </row>
     <row r="82" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5469,11 +5241,11 @@
       <c r="C82" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D82" s="22" t="s">
-        <v>320</v>
+      <c r="D82" s="29">
+        <v>44.9</v>
       </c>
       <c r="E82" s="21" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
     </row>
     <row r="83" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5483,11 +5255,11 @@
       <c r="C83" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D83" s="22" t="s">
-        <v>318</v>
+      <c r="D83" s="29">
+        <v>43.81</v>
       </c>
       <c r="E83" s="21" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
     </row>
     <row r="84" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5497,11 +5269,11 @@
       <c r="C84" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D84" s="22" t="s">
-        <v>316</v>
+      <c r="D84" s="29">
+        <v>44.19</v>
       </c>
       <c r="E84" s="21" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
     </row>
     <row r="85" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5511,11 +5283,11 @@
       <c r="C85" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D85" s="22" t="s">
-        <v>314</v>
+      <c r="D85" s="29">
+        <v>43.55</v>
       </c>
       <c r="E85" s="21" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
     </row>
     <row r="86" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5525,11 +5297,11 @@
       <c r="C86" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D86" s="22" t="s">
-        <v>312</v>
+      <c r="D86" s="29">
+        <v>42.84</v>
       </c>
       <c r="E86" s="21" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="87" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5539,11 +5311,11 @@
       <c r="C87" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="D87" s="22" t="s">
-        <v>310</v>
+      <c r="D87" s="29">
+        <v>42.61</v>
       </c>
       <c r="E87" s="21" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="88" spans="2:5" ht="15" x14ac:dyDescent="0.25">
@@ -5551,17 +5323,18 @@
         <v>160</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="D88" s="22" t="s">
-        <v>308</v>
+        <v>387</v>
+      </c>
+      <c r="D88" s="29">
+        <v>43.49</v>
       </c>
       <c r="E88" s="21" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5657,10 +5430,10 @@
       <c r="F2" s="7">
         <v>6</v>
       </c>
-      <c r="G2" s="27" t="s">
+      <c r="G2" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H2" s="28"/>
+      <c r="H2" s="25"/>
       <c r="I2" s="13" t="s">
         <v>215</v>
       </c>
@@ -5679,10 +5452,10 @@
       <c r="N2" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="O2" s="27" t="s">
+      <c r="O2" s="24" t="s">
         <v>219</v>
       </c>
-      <c r="P2" s="28"/>
+      <c r="P2" s="25"/>
       <c r="Q2" s="13"/>
       <c r="R2" s="7">
         <v>2005</v>
@@ -5708,10 +5481,10 @@
       <c r="F3" s="15">
         <v>6</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="H3" s="26"/>
+      <c r="H3" s="27"/>
       <c r="I3" s="16" t="s">
         <v>221</v>
       </c>
@@ -5757,10 +5530,10 @@
       <c r="F4" s="7">
         <v>7</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H4" s="28"/>
+      <c r="H4" s="25"/>
       <c r="I4" s="13" t="s">
         <v>224</v>
       </c>
@@ -5802,10 +5575,10 @@
       <c r="F5" s="7">
         <v>7</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="G5" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H5" s="28"/>
+      <c r="H5" s="25"/>
       <c r="I5" s="13" t="s">
         <v>225</v>
       </c>
@@ -5847,10 +5620,10 @@
       <c r="F6" s="7">
         <v>7</v>
       </c>
-      <c r="G6" s="27" t="s">
+      <c r="G6" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H6" s="28"/>
+      <c r="H6" s="25"/>
       <c r="I6" s="13" t="s">
         <v>225</v>
       </c>
@@ -5892,10 +5665,10 @@
       <c r="F7" s="7">
         <v>7</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="G7" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H7" s="28"/>
+      <c r="H7" s="25"/>
       <c r="I7" s="13" t="s">
         <v>225</v>
       </c>
@@ -5917,11 +5690,11 @@
       <c r="O7" s="7">
         <v>10</v>
       </c>
-      <c r="P7" s="27" t="s">
+      <c r="P7" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="Q7" s="28"/>
-      <c r="R7" s="28"/>
+      <c r="Q7" s="25"/>
+      <c r="R7" s="25"/>
       <c r="S7" s="13"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
@@ -5939,10 +5712,10 @@
       <c r="F8" s="7">
         <v>7</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H8" s="28"/>
+      <c r="H8" s="25"/>
       <c r="I8" s="13" t="s">
         <v>225</v>
       </c>
@@ -5984,10 +5757,10 @@
       <c r="F9" s="7">
         <v>8</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="G9" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H9" s="28"/>
+      <c r="H9" s="25"/>
       <c r="I9" s="13" t="s">
         <v>215</v>
       </c>
@@ -6009,11 +5782,11 @@
       <c r="O9" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="P9" s="27" t="s">
+      <c r="P9" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="Q9" s="28"/>
-      <c r="R9" s="28"/>
+      <c r="Q9" s="25"/>
+      <c r="R9" s="25"/>
       <c r="S9" s="13"/>
     </row>
     <row r="10" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6033,10 +5806,10 @@
       <c r="F10" s="7">
         <v>8</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="G10" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H10" s="28"/>
+      <c r="H10" s="25"/>
       <c r="I10" s="13" t="s">
         <v>230</v>
       </c>
@@ -6058,10 +5831,10 @@
       <c r="O10" s="7">
         <v>10</v>
       </c>
-      <c r="P10" s="27" t="s">
+      <c r="P10" s="24" t="s">
         <v>232</v>
       </c>
-      <c r="Q10" s="28"/>
+      <c r="Q10" s="25"/>
       <c r="R10" s="7">
         <v>2005</v>
       </c>
@@ -6234,12 +6007,12 @@
       </c>
       <c r="N14" s="13"/>
       <c r="O14" s="13"/>
-      <c r="P14" s="27" t="s">
+      <c r="P14" s="24" t="s">
         <v>239</v>
       </c>
-      <c r="Q14" s="28"/>
-      <c r="R14" s="28"/>
-      <c r="S14" s="28"/>
+      <c r="Q14" s="25"/>
+      <c r="R14" s="25"/>
+      <c r="S14" s="25"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
@@ -6277,12 +6050,12 @@
       </c>
       <c r="N15" s="13"/>
       <c r="O15" s="13"/>
-      <c r="P15" s="27" t="s">
+      <c r="P15" s="24" t="s">
         <v>240</v>
       </c>
-      <c r="Q15" s="28"/>
-      <c r="R15" s="28"/>
-      <c r="S15" s="28"/>
+      <c r="Q15" s="25"/>
+      <c r="R15" s="25"/>
+      <c r="S15" s="25"/>
     </row>
     <row r="16" spans="1:19" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7">
@@ -6449,12 +6222,12 @@
       </c>
       <c r="N19" s="13"/>
       <c r="O19" s="13"/>
-      <c r="P19" s="27" t="s">
+      <c r="P19" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="Q19" s="28"/>
-      <c r="R19" s="28"/>
-      <c r="S19" s="28"/>
+      <c r="Q19" s="25"/>
+      <c r="R19" s="25"/>
+      <c r="S19" s="25"/>
     </row>
     <row r="20" spans="1:19" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7">
@@ -6621,11 +6394,11 @@
       </c>
       <c r="N23" s="13"/>
       <c r="O23" s="13"/>
-      <c r="P23" s="27" t="s">
+      <c r="P23" s="24" t="s">
         <v>244</v>
       </c>
-      <c r="Q23" s="28"/>
-      <c r="R23" s="28"/>
+      <c r="Q23" s="25"/>
+      <c r="R23" s="25"/>
       <c r="S23" s="13"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
@@ -6774,10 +6547,10 @@
       <c r="F27" s="7">
         <v>55</v>
       </c>
-      <c r="G27" s="27" t="s">
+      <c r="G27" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H27" s="28"/>
+      <c r="H27" s="25"/>
       <c r="I27" s="13" t="s">
         <v>245</v>
       </c>
@@ -6827,10 +6600,10 @@
       <c r="F28" s="7">
         <v>8</v>
       </c>
-      <c r="G28" s="27" t="s">
+      <c r="G28" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H28" s="28"/>
+      <c r="H28" s="25"/>
       <c r="I28" s="13" t="s">
         <v>249</v>
       </c>
@@ -6874,10 +6647,10 @@
       <c r="F29" s="15">
         <v>55</v>
       </c>
-      <c r="G29" s="25" t="s">
+      <c r="G29" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="H29" s="26"/>
+      <c r="H29" s="27"/>
       <c r="I29" s="16" t="s">
         <v>254</v>
       </c>
@@ -6923,10 +6696,10 @@
       <c r="F30" s="7">
         <v>8</v>
       </c>
-      <c r="G30" s="27" t="s">
+      <c r="G30" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H30" s="28"/>
+      <c r="H30" s="25"/>
       <c r="I30" s="13" t="s">
         <v>258</v>
       </c>
@@ -7032,12 +6805,12 @@
       </c>
       <c r="N32" s="13"/>
       <c r="O32" s="13"/>
-      <c r="P32" s="27" t="s">
+      <c r="P32" s="24" t="s">
         <v>264</v>
       </c>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
+      <c r="Q32" s="25"/>
+      <c r="R32" s="25"/>
+      <c r="S32" s="25"/>
     </row>
     <row r="33" spans="1:19" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7">
@@ -7075,12 +6848,12 @@
       </c>
       <c r="N33" s="13"/>
       <c r="O33" s="13"/>
-      <c r="P33" s="27" t="s">
+      <c r="P33" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="Q33" s="28"/>
-      <c r="R33" s="28"/>
-      <c r="S33" s="28"/>
+      <c r="Q33" s="25"/>
+      <c r="R33" s="25"/>
+      <c r="S33" s="25"/>
     </row>
     <row r="34" spans="1:19" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7">
@@ -7400,10 +7173,10 @@
       <c r="F41" s="7">
         <v>6</v>
       </c>
-      <c r="G41" s="27" t="s">
+      <c r="G41" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H41" s="28"/>
+      <c r="H41" s="25"/>
       <c r="I41" s="13" t="s">
         <v>267</v>
       </c>
@@ -7445,10 +7218,10 @@
       <c r="F42" s="7">
         <v>6</v>
       </c>
-      <c r="G42" s="27" t="s">
+      <c r="G42" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H42" s="28"/>
+      <c r="H42" s="25"/>
       <c r="I42" s="13" t="s">
         <v>269</v>
       </c>
@@ -7492,10 +7265,10 @@
       <c r="F43" s="15">
         <v>55</v>
       </c>
-      <c r="G43" s="25" t="s">
+      <c r="G43" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="H43" s="26"/>
+      <c r="H43" s="27"/>
       <c r="I43" s="16" t="s">
         <v>270</v>
       </c>
@@ -7541,10 +7314,10 @@
       <c r="F44" s="7">
         <v>8</v>
       </c>
-      <c r="G44" s="27" t="s">
+      <c r="G44" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H44" s="28"/>
+      <c r="H44" s="25"/>
       <c r="I44" s="13" t="s">
         <v>269</v>
       </c>
@@ -7566,12 +7339,12 @@
       <c r="O44" s="7">
         <v>10</v>
       </c>
-      <c r="P44" s="27" t="s">
+      <c r="P44" s="24" t="s">
         <v>272</v>
       </c>
-      <c r="Q44" s="28"/>
-      <c r="R44" s="28"/>
-      <c r="S44" s="28"/>
+      <c r="Q44" s="25"/>
+      <c r="R44" s="25"/>
+      <c r="S44" s="25"/>
     </row>
     <row r="45" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="15">
@@ -7590,10 +7363,10 @@
       <c r="F45" s="15">
         <v>6</v>
       </c>
-      <c r="G45" s="25" t="s">
+      <c r="G45" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="H45" s="26"/>
+      <c r="H45" s="27"/>
       <c r="I45" s="16" t="s">
         <v>273</v>
       </c>
@@ -7639,10 +7412,10 @@
       <c r="F46" s="7">
         <v>55</v>
       </c>
-      <c r="G46" s="27" t="s">
+      <c r="G46" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H46" s="28"/>
+      <c r="H46" s="25"/>
       <c r="I46" s="13" t="s">
         <v>276</v>
       </c>
@@ -7684,10 +7457,10 @@
       <c r="F47" s="7">
         <v>8</v>
       </c>
-      <c r="G47" s="27" t="s">
+      <c r="G47" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H47" s="28"/>
+      <c r="H47" s="25"/>
       <c r="I47" s="13" t="s">
         <v>276</v>
       </c>
@@ -7729,10 +7502,10 @@
       <c r="F48" s="7">
         <v>55</v>
       </c>
-      <c r="G48" s="27" t="s">
+      <c r="G48" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H48" s="28"/>
+      <c r="H48" s="25"/>
       <c r="I48" s="13" t="s">
         <v>277</v>
       </c>
@@ -7750,11 +7523,11 @@
       </c>
       <c r="N48" s="13"/>
       <c r="O48" s="13"/>
-      <c r="P48" s="27" t="s">
+      <c r="P48" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="Q48" s="28"/>
-      <c r="R48" s="28"/>
+      <c r="Q48" s="25"/>
+      <c r="R48" s="25"/>
       <c r="S48" s="13"/>
     </row>
     <row r="49" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7774,10 +7547,10 @@
       <c r="F49" s="15">
         <v>7</v>
       </c>
-      <c r="G49" s="25" t="s">
+      <c r="G49" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="H49" s="26"/>
+      <c r="H49" s="27"/>
       <c r="I49" s="16" t="s">
         <v>280</v>
       </c>
@@ -7799,10 +7572,10 @@
       <c r="O49" s="15">
         <v>5</v>
       </c>
-      <c r="P49" s="25" t="s">
+      <c r="P49" s="26" t="s">
         <v>283</v>
       </c>
-      <c r="Q49" s="26"/>
+      <c r="Q49" s="27"/>
       <c r="R49" s="15">
         <v>2005</v>
       </c>
@@ -7825,10 +7598,10 @@
       <c r="F50" s="7">
         <v>55</v>
       </c>
-      <c r="G50" s="27" t="s">
+      <c r="G50" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H50" s="28"/>
+      <c r="H50" s="25"/>
       <c r="I50" s="13" t="s">
         <v>284</v>
       </c>
@@ -7850,10 +7623,10 @@
       <c r="O50" s="7">
         <v>6</v>
       </c>
-      <c r="P50" s="27" t="s">
+      <c r="P50" s="24" t="s">
         <v>289</v>
       </c>
-      <c r="Q50" s="28"/>
+      <c r="Q50" s="25"/>
       <c r="R50" s="13"/>
       <c r="S50" s="13"/>
     </row>
@@ -7874,10 +7647,10 @@
       <c r="F51" s="7">
         <v>6</v>
       </c>
-      <c r="G51" s="27" t="s">
+      <c r="G51" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H51" s="28"/>
+      <c r="H51" s="25"/>
       <c r="I51" s="13" t="s">
         <v>290</v>
       </c>
@@ -7923,10 +7696,10 @@
       <c r="F52" s="15">
         <v>7</v>
       </c>
-      <c r="G52" s="25" t="s">
+      <c r="G52" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="H52" s="26"/>
+      <c r="H52" s="27"/>
       <c r="I52" s="16" t="s">
         <v>296</v>
       </c>
@@ -8291,10 +8064,10 @@
       <c r="F60" s="7">
         <v>8</v>
       </c>
-      <c r="G60" s="27" t="s">
+      <c r="G60" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="H60" s="28"/>
+      <c r="H60" s="25"/>
       <c r="I60" s="13" t="s">
         <v>304</v>
       </c>
@@ -9280,32 +9053,6 @@
     </filterColumn>
   </autoFilter>
   <mergeCells count="40">
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="P7:R7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="P33:S33"/>
-    <mergeCell ref="P44:S44"/>
-    <mergeCell ref="P48:R48"/>
-    <mergeCell ref="P49:Q49"/>
-    <mergeCell ref="P50:Q50"/>
-    <mergeCell ref="P9:R9"/>
-    <mergeCell ref="P10:Q10"/>
-    <mergeCell ref="P14:S14"/>
-    <mergeCell ref="P15:S15"/>
-    <mergeCell ref="P19:S19"/>
-    <mergeCell ref="P23:R23"/>
-    <mergeCell ref="P32:S32"/>
     <mergeCell ref="G52:H52"/>
     <mergeCell ref="G60:H60"/>
     <mergeCell ref="G30:H30"/>
@@ -9320,6 +9067,32 @@
     <mergeCell ref="G49:H49"/>
     <mergeCell ref="G50:H50"/>
     <mergeCell ref="G51:H51"/>
+    <mergeCell ref="P44:S44"/>
+    <mergeCell ref="P48:R48"/>
+    <mergeCell ref="P49:Q49"/>
+    <mergeCell ref="P50:Q50"/>
+    <mergeCell ref="P9:R9"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="P14:S14"/>
+    <mergeCell ref="P15:S15"/>
+    <mergeCell ref="P19:S19"/>
+    <mergeCell ref="P23:R23"/>
+    <mergeCell ref="P32:S32"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="P33:S33"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -9328,12 +9101,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ada196f1-b314-4482-a04c-235b25854a0d" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ad035cd5-bf96-4d76-9017-fe4affe7c009">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9572,20 +9347,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ada196f1-b314-4482-a04c-235b25854a0d" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ad035cd5-bf96-4d76-9017-fe4affe7c009">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1194C2B7-4BD7-4B07-93FB-838972F49667}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF6E2962-8215-480F-B58A-1690525584CB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="ada196f1-b314-4482-a04c-235b25854a0d"/>
+    <ds:schemaRef ds:uri="ad035cd5-bf96-4d76-9017-fe4affe7c009"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9610,18 +9392,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF6E2962-8215-480F-B58A-1690525584CB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1194C2B7-4BD7-4B07-93FB-838972F49667}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="ada196f1-b314-4482-a04c-235b25854a0d"/>
-    <ds:schemaRef ds:uri="ad035cd5-bf96-4d76-9017-fe4affe7c009"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>